<commit_message>
feat(catalogo): códigos agrupados partidos en incisos (S2 25(a)(i)–(v), S1 44(a)(i)–(v), S2 36(a)–(d), S2 36(e)(i)–(iv)) — PREPARADA, NO APLICADA
Migración de datos idempotente y aditiva (18 filas, enlaces de solicitudes y plantilla), seed, poblar-demo,
bloques 27 y 40, Anexo A, auditoría del catálogo con la lista para revisión de Esteban, y 18 filas en la hoja
de taxonomía de la plantilla Excel (diferencia esperada en el próximo despliegue).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/taxonomia-base.xlsx
+++ b/assets/taxonomia-base.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="371">
   <si>
     <t>Sección</t>
   </si>
@@ -217,6 +217,21 @@
   </si>
   <si>
     <t>NIIF S1 44 (a)(i)a(v)</t>
+  </si>
+  <si>
+    <t>NIIF S1 44 (a)(i)</t>
+  </si>
+  <si>
+    <t>NIIF S1 44 (a)(ii)</t>
+  </si>
+  <si>
+    <t>NIIF S1 44 (a)(iii)</t>
+  </si>
+  <si>
+    <t>NIIF S1 44 (a)(iv)</t>
+  </si>
+  <si>
+    <t>NIIF S1 44 (a)(v)</t>
   </si>
   <si>
     <t>NIIF S1 44 (a)(vi)</t>
@@ -411,6 +426,21 @@
 (iv) si la entidad da prioridad a los riesgos relacionados con el clima en relación con otros tipos de riesgo y cómo lo hace;
 (v) cómo supervisa la entidad los riesgos relacionados con el clima; y
 </t>
+  </si>
+  <si>
+    <t>NIIF S2 25 (a)(i)</t>
+  </si>
+  <si>
+    <t>NIIF S2 25 (a)(ii)</t>
+  </si>
+  <si>
+    <t>NIIF S2 25 (a)(iii)</t>
+  </si>
+  <si>
+    <t>NIIF S2 25 (a)(iv)</t>
+  </si>
+  <si>
+    <t>NIIF S2 25 (a)(v)</t>
   </si>
   <si>
     <t>NIIF S2 25 (a)(vi)</t>
@@ -856,6 +886,18 @@
     <t>NIIF S2 36 (a)a(d)</t>
   </si>
   <si>
+    <t>NIIF S2 36 (a)</t>
+  </si>
+  <si>
+    <t>NIIF S2 36 (b)</t>
+  </si>
+  <si>
+    <t>NIIF S2 36 (c)</t>
+  </si>
+  <si>
+    <t>NIIF S2 36 (d)</t>
+  </si>
+  <si>
     <t>NIIF S2 36 (e)(i)a(iv)</t>
   </si>
   <si>
@@ -863,6 +905,18 @@
   </si>
   <si>
     <t>Si</t>
+  </si>
+  <si>
+    <t>NIIF S2 36 (e)(i)</t>
+  </si>
+  <si>
+    <t>NIIF S2 36 (e)(ii)</t>
+  </si>
+  <si>
+    <t>NIIF S2 36 (e)(iii)</t>
+  </si>
+  <si>
+    <t>NIIF S2 36 (e)(iv)</t>
   </si>
   <si>
     <t>Contenidos temáticos -Empleo</t>
@@ -3103,7 +3157,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="76" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
       <c r="B1" s="76"/>
       <c r="C1" s="76"/>
@@ -3118,13 +3172,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="D2" s="82"/>
       <c r="E2" s="82"/>
@@ -3156,24 +3210,24 @@
       <c r="A4" s="66"/>
       <c r="B4" s="66"/>
       <c r="C4" s="83" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="D4" s="83" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="E4" s="83" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="F4" s="66"/>
       <c r="G4" s="66"/>
       <c r="H4" s="83" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="I4" s="83" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="J4" s="83" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="K4" s="66"/>
     </row>
@@ -3339,7 +3393,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="76" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="B1" s="76"/>
       <c r="C1" s="76"/>
@@ -3354,13 +3408,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="D2" s="82"/>
       <c r="E2" s="82"/>
@@ -3392,24 +3446,24 @@
       <c r="A4" s="66"/>
       <c r="B4" s="66"/>
       <c r="C4" s="83" t="s">
-        <v>316</v>
+        <v>334</v>
       </c>
       <c r="D4" s="83" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="E4" s="83" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="F4" s="66"/>
       <c r="G4" s="66"/>
       <c r="H4" s="83" t="s">
-        <v>316</v>
+        <v>334</v>
       </c>
       <c r="I4" s="83" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="J4" s="83" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="K4" s="66"/>
     </row>
@@ -3653,7 +3707,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="76" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
       <c r="B1" s="76"/>
       <c r="C1" s="76"/>
@@ -3668,13 +3722,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>319</v>
+        <v>337</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
       <c r="D2" s="82"/>
       <c r="E2" s="82"/>
@@ -3706,24 +3760,24 @@
       <c r="A4" s="66"/>
       <c r="B4" s="66"/>
       <c r="C4" s="83" t="s">
-        <v>322</v>
+        <v>340</v>
       </c>
       <c r="D4" s="83" t="s">
-        <v>323</v>
+        <v>341</v>
       </c>
       <c r="E4" s="83" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="F4" s="66"/>
       <c r="G4" s="66"/>
       <c r="H4" s="83" t="s">
-        <v>324</v>
+        <v>342</v>
       </c>
       <c r="I4" s="83" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
       <c r="J4" s="83" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="K4" s="66"/>
     </row>
@@ -3968,7 +4022,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
-        <v>326</v>
+        <v>344</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -3983,37 +4037,37 @@
     </row>
     <row r="2" ht="70" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="E2" s="64" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="F2" s="64" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="G2" s="64" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="H2" s="64" t="s">
-        <v>288</v>
+        <v>306</v>
       </c>
       <c r="I2" s="64" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="J2" s="64" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
       <c r="K2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -4143,7 +4197,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -4153,22 +4207,22 @@
     </row>
     <row r="2" ht="65" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="E2" s="64" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="F2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -4255,7 +4309,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -4263,16 +4317,16 @@
     </row>
     <row r="2" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4346,7 +4400,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="76" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
       <c r="B1" s="76"/>
       <c r="C1" s="76"/>
@@ -4356,22 +4410,22 @@
     </row>
     <row r="2" ht="80" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
       <c r="E2" s="64" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="F2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -4459,7 +4513,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="76" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
       <c r="B1" s="76"/>
       <c r="C1" s="76"/>
@@ -4467,21 +4521,21 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>298</v>
+        <v>316</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="69" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="B3" s="66"/>
       <c r="C3" s="66"/>
@@ -4489,7 +4543,7 @@
     </row>
     <row r="4" ht="110" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="69" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="B4" s="66"/>
       <c r="C4" s="66"/>
@@ -4497,7 +4551,7 @@
     </row>
     <row r="5" ht="110" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="69" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
       <c r="B5" s="66"/>
       <c r="C5" s="66"/>
@@ -4505,7 +4559,7 @@
     </row>
     <row r="6" ht="110" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="69" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="B6" s="66"/>
       <c r="C6" s="66"/>
@@ -4513,7 +4567,7 @@
     </row>
     <row r="7" ht="110" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="69" t="s">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="B7" s="66"/>
       <c r="C7" s="66"/>
@@ -4529,7 +4583,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D383"/>
+  <dimension ref="A1:D401"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="9.1640625"/>
   <cols>
     <col min="1" max="1" width="31.6640625" style="1" hidden="1" customWidth="1"/>
@@ -4915,26 +4969,24 @@
     </row>
     <row r="44" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="18"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>21</v>
-      </c>
+      <c r="B44" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" s="15"/>
+      <c r="D44" s="10"/>
     </row>
     <row r="45" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="18"/>
-      <c r="B45" s="11"/>
+      <c r="B45" s="11" t="s">
+        <v>53</v>
+      </c>
       <c r="C45" s="15"/>
-      <c r="D45" s="10" t="s">
-        <v>52</v>
-      </c>
+      <c r="D45" s="10"/>
     </row>
     <row r="46" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="18"/>
       <c r="B46" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C46" s="15"/>
       <c r="D46" s="10"/>
@@ -4942,136 +4994,134 @@
     <row r="47" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="18"/>
       <c r="B47" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C47" s="15" t="s">
-        <v>40</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="C47" s="15"/>
       <c r="D47" s="10"/>
     </row>
     <row r="48" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="18"/>
-      <c r="B48" s="14"/>
+      <c r="B48" s="11" t="s">
+        <v>56</v>
+      </c>
       <c r="C48" s="15"/>
-      <c r="D48" s="16" t="s">
-        <v>55</v>
-      </c>
+      <c r="D48" s="10"/>
     </row>
     <row r="49" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="18"/>
-      <c r="B49" s="14"/>
+      <c r="B49" s="11"/>
       <c r="C49" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D49" s="16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="50" ht="396" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="50" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="18"/>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="11"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C50" s="15"/>
-      <c r="D50" s="10"/>
     </row>
     <row r="51" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="18"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="D51" s="16" t="s">
+      <c r="B51" s="11" t="s">
         <v>58</v>
       </c>
+      <c r="C51" s="15"/>
+      <c r="D51" s="10"/>
     </row>
     <row r="52" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="18"/>
-      <c r="B52" s="12" t="s">
+      <c r="B52" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C52" s="15"/>
-      <c r="D52" s="20"/>
-    </row>
-    <row r="53" ht="297" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C52" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D52" s="10"/>
+    </row>
+    <row r="53" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="18"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="D53" s="10"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="16" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="54" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="18"/>
       <c r="B54" s="14"/>
-      <c r="C54" s="15"/>
+      <c r="C54" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="D54" s="16" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="55" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" ht="396" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="18"/>
       <c r="B55" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D55" s="14"/>
+        <v>62</v>
+      </c>
+      <c r="C55" s="15"/>
+      <c r="D55" s="10"/>
     </row>
     <row r="56" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="18"/>
-      <c r="B56" s="11"/>
+      <c r="B56" s="14"/>
       <c r="C56" s="15" t="s">
         <v>40</v>
       </c>
       <c r="D56" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="57" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="18"/>
-      <c r="B57" s="11" t="s">
-        <v>63</v>
+      <c r="B57" s="12" t="s">
+        <v>64</v>
       </c>
       <c r="C57" s="15"/>
-      <c r="D57" s="10"/>
-    </row>
-    <row r="58" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D57" s="20"/>
+    </row>
+    <row r="58" ht="297" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="18"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="16" t="s">
-        <v>64</v>
-      </c>
+      <c r="B58" s="12"/>
+      <c r="C58" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D58" s="10"/>
     </row>
     <row r="59" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="18"/>
-      <c r="B59" s="11" t="s">
+      <c r="B59" s="14"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="C59" s="15" t="s">
+    </row>
+    <row r="60" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="18"/>
+      <c r="B60" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C60" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D59" s="10"/>
-    </row>
-    <row r="60" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="18"/>
-      <c r="B60" s="21"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="16" t="s">
-        <v>66</v>
-      </c>
+      <c r="D60" s="14"/>
     </row>
     <row r="61" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="18"/>
-      <c r="B61" s="11" t="s">
-        <v>67</v>
-      </c>
+      <c r="B61" s="11"/>
       <c r="C61" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D61" s="14"/>
+      <c r="D61" s="16" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="62" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="18"/>
@@ -5079,78 +5129,76 @@
         <v>68</v>
       </c>
       <c r="C62" s="15"/>
-      <c r="D62" s="14"/>
+      <c r="D62" s="10"/>
     </row>
     <row r="63" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="18"/>
-      <c r="B63" s="11" t="s">
+      <c r="B63" s="11"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="C63" s="15"/>
-      <c r="D63" s="14"/>
-    </row>
-    <row r="64" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="18"/>
       <c r="B64" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="C64" s="15"/>
-      <c r="D64" s="14"/>
-    </row>
-    <row r="65" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C64" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D64" s="10"/>
+    </row>
+    <row r="65" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="18"/>
-      <c r="B65" s="12" t="s">
+      <c r="B65" s="21"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="C65" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D65" s="14"/>
     </row>
     <row r="66" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="18"/>
-      <c r="B66" s="12"/>
-      <c r="C66" s="15"/>
-      <c r="D66" s="14" t="s">
-        <v>13</v>
-      </c>
+      <c r="B66" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C66" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D66" s="14"/>
     </row>
     <row r="67" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="18"/>
-      <c r="B67" s="12"/>
+      <c r="B67" s="11" t="s">
+        <v>73</v>
+      </c>
       <c r="C67" s="15"/>
-      <c r="D67" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="68" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="B68" s="12"/>
-      <c r="C68" s="7" t="s">
+      <c r="D67" s="14"/>
+    </row>
+    <row r="68" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="18"/>
+      <c r="B68" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="D68" s="10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="69" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C68" s="15"/>
+      <c r="D68" s="14"/>
+    </row>
+    <row r="69" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="18"/>
       <c r="B69" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="C69" s="15" t="s">
-        <v>40</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="C69" s="15"/>
       <c r="D69" s="14"/>
     </row>
     <row r="70" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="18"/>
       <c r="B70" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C70" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="C70" s="15"/>
       <c r="D70" s="14"/>
     </row>
     <row r="71" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5158,7 +5206,7 @@
       <c r="B71" s="12"/>
       <c r="C71" s="15"/>
       <c r="D71" s="14" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="72" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5166,114 +5214,120 @@
       <c r="B72" s="12"/>
       <c r="C72" s="15"/>
       <c r="D72" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="18" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="73" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="18"/>
-      <c r="B73" s="12" t="s">
+      <c r="B73" s="12"/>
+      <c r="C73" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C73" s="15"/>
-      <c r="D73" s="14"/>
+      <c r="D73" s="10" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="74" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="18"/>
-      <c r="B74" s="12"/>
-      <c r="C74" s="15"/>
-      <c r="D74" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="75" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B74" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C74" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D74" s="14"/>
+    </row>
+    <row r="75" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="18"/>
-      <c r="B75" s="12"/>
+      <c r="B75" s="12" t="s">
+        <v>82</v>
+      </c>
       <c r="C75" s="15"/>
-      <c r="D75" s="10" t="s">
-        <v>22</v>
-      </c>
+      <c r="D75" s="14"/>
     </row>
     <row r="76" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="18"/>
-      <c r="B76" s="14"/>
+      <c r="B76" s="12"/>
       <c r="C76" s="15"/>
-      <c r="D76" s="16" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="77" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D76" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="18"/>
-      <c r="B77" s="14"/>
+      <c r="B77" s="12"/>
       <c r="C77" s="15"/>
-      <c r="D77" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="78" ht="307" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D77" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="78" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="18"/>
-      <c r="B78" s="14" t="s">
-        <v>82</v>
+      <c r="B78" s="12" t="s">
+        <v>84</v>
       </c>
       <c r="C78" s="15"/>
-      <c r="D78" s="10"/>
+      <c r="D78" s="14"/>
     </row>
     <row r="79" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="18"/>
-      <c r="B79" s="11" t="s">
-        <v>83</v>
-      </c>
+      <c r="B79" s="12"/>
       <c r="C79" s="15"/>
-      <c r="D79" s="14"/>
+      <c r="D79" s="10" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="80" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="18"/>
-      <c r="B80" s="11"/>
+      <c r="B80" s="12"/>
       <c r="C80" s="15"/>
-      <c r="D80" s="16" t="s">
-        <v>28</v>
+      <c r="D80" s="10" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="81" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="18"/>
-      <c r="B81" s="11" t="s">
-        <v>84</v>
-      </c>
+      <c r="B81" s="14"/>
       <c r="C81" s="15"/>
-      <c r="D81" s="14"/>
-    </row>
-    <row r="82" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D81" s="16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="82" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="18"/>
-      <c r="B82" s="11" t="s">
-        <v>85</v>
-      </c>
+      <c r="B82" s="14"/>
       <c r="C82" s="15"/>
-      <c r="D82" s="14"/>
-    </row>
-    <row r="83" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D82" s="22" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="83" ht="307" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="18"/>
-      <c r="B83" s="11"/>
+      <c r="B83" s="14" t="s">
+        <v>87</v>
+      </c>
       <c r="C83" s="15"/>
-      <c r="D83" s="16" t="s">
-        <v>86</v>
-      </c>
+      <c r="D83" s="10"/>
     </row>
     <row r="84" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="18"/>
       <c r="B84" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C84" s="15"/>
       <c r="D84" s="14"/>
     </row>
-    <row r="85" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="18"/>
-      <c r="B85" s="11" t="s">
-        <v>88</v>
-      </c>
+      <c r="B85" s="11"/>
       <c r="C85" s="15"/>
-      <c r="D85" s="14"/>
-    </row>
-    <row r="86" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D85" s="16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="86" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="18"/>
       <c r="B86" s="11" t="s">
         <v>89</v>
@@ -5289,21 +5343,21 @@
       <c r="C87" s="15"/>
       <c r="D87" s="14"/>
     </row>
-    <row r="88" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="18"/>
-      <c r="B88" s="11" t="s">
+      <c r="B88" s="11"/>
+      <c r="C88" s="15"/>
+      <c r="D88" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C88" s="15"/>
-      <c r="D88" s="14"/>
-    </row>
-    <row r="89" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="18"/>
       <c r="B89" s="11" t="s">
         <v>92</v>
       </c>
       <c r="C89" s="15"/>
-      <c r="D89" s="23"/>
+      <c r="D89" s="14"/>
     </row>
     <row r="90" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="18"/>
@@ -5311,139 +5365,139 @@
         <v>93</v>
       </c>
       <c r="C90" s="15"/>
-      <c r="D90" s="23"/>
-    </row>
-    <row r="91" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D90" s="14"/>
+    </row>
+    <row r="91" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="18"/>
-      <c r="B91" s="11"/>
-      <c r="C91" s="7"/>
-      <c r="D91" s="16" t="s">
-        <v>34</v>
-      </c>
+      <c r="B91" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C91" s="15"/>
+      <c r="D91" s="14"/>
     </row>
     <row r="92" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B92" s="11"/>
+      <c r="A92" s="18"/>
+      <c r="B92" s="11" t="s">
+        <v>95</v>
+      </c>
       <c r="C92" s="15"/>
-      <c r="D92" s="17" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="93" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="5"/>
+      <c r="D92" s="14"/>
+    </row>
+    <row r="93" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="18"/>
       <c r="B93" s="11" t="s">
         <v>96</v>
       </c>
       <c r="C93" s="15"/>
       <c r="D93" s="14"/>
     </row>
-    <row r="94" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="5"/>
+    <row r="94" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="18"/>
       <c r="B94" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C94" s="15"/>
-      <c r="D94" s="14" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="95" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="5"/>
+      <c r="D94" s="23"/>
+    </row>
+    <row r="95" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" s="18"/>
       <c r="B95" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C95" s="15"/>
-      <c r="D95" s="14" t="s">
-        <v>98</v>
-      </c>
+      <c r="D95" s="23"/>
     </row>
     <row r="96" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="5"/>
+      <c r="A96" s="18"/>
       <c r="B96" s="11"/>
-      <c r="C96" s="15"/>
-      <c r="D96" s="17" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="97" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="24" t="s">
+      <c r="C96" s="7"/>
+      <c r="D96" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="97" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B97" s="25" t="s">
+      <c r="B97" s="11"/>
+      <c r="C97" s="15"/>
+      <c r="D97" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C97" s="15"/>
-      <c r="D97" s="14"/>
-    </row>
-    <row r="98" ht="51" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="24"/>
+    </row>
+    <row r="98" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="5"/>
       <c r="B98" s="11" t="s">
         <v>101</v>
       </c>
       <c r="C98" s="15"/>
       <c r="D98" s="14"/>
     </row>
-    <row r="99" ht="75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="24"/>
-      <c r="B99" s="11"/>
+    <row r="99" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="5"/>
+      <c r="B99" s="11" t="s">
+        <v>101</v>
+      </c>
       <c r="C99" s="15"/>
-      <c r="D99" s="10"/>
+      <c r="D99" s="14" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="100" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="24"/>
+      <c r="A100" s="5"/>
       <c r="B100" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C100" s="15"/>
-      <c r="D100" s="14"/>
-    </row>
-    <row r="101" ht="78" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="24"/>
+      <c r="D100" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="101" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" s="5"/>
       <c r="B101" s="11"/>
       <c r="C101" s="15"/>
-      <c r="D101" s="10"/>
-    </row>
-    <row r="102" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="24"/>
-      <c r="B102" s="11" t="s">
-        <v>102</v>
+      <c r="D101" s="17" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="102" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" s="25" t="s">
+        <v>105</v>
       </c>
       <c r="C102" s="15"/>
-      <c r="D102" s="14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="103" ht="75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D102" s="14"/>
+    </row>
+    <row r="103" ht="51" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="24"/>
-      <c r="B103" s="11"/>
+      <c r="B103" s="11" t="s">
+        <v>106</v>
+      </c>
       <c r="C103" s="15"/>
-      <c r="D103" s="10"/>
-    </row>
-    <row r="104" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D103" s="14"/>
+    </row>
+    <row r="104" ht="75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="24"/>
-      <c r="B104" s="14"/>
+      <c r="B104" s="11"/>
       <c r="C104" s="15"/>
-      <c r="D104" s="16" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="105" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D104" s="10"/>
+    </row>
+    <row r="105" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="24"/>
-      <c r="B105" s="14" t="s">
-        <v>105</v>
+      <c r="B105" s="11" t="s">
+        <v>107</v>
       </c>
       <c r="C105" s="15"/>
-      <c r="D105" s="23"/>
-    </row>
-    <row r="106" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D105" s="14"/>
+    </row>
+    <row r="106" ht="78" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="24"/>
-      <c r="B106" s="14" t="s">
-        <v>106</v>
-      </c>
+      <c r="B106" s="11"/>
       <c r="C106" s="15"/>
-      <c r="D106" s="23"/>
+      <c r="D106" s="10"/>
     </row>
     <row r="107" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="24"/>
@@ -5451,456 +5505,454 @@
         <v>107</v>
       </c>
       <c r="C107" s="15"/>
-      <c r="D107" s="10"/>
-    </row>
-    <row r="108" ht="65" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D107" s="14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="108" ht="75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="24"/>
       <c r="B108" s="11"/>
       <c r="C108" s="15"/>
       <c r="D108" s="10"/>
     </row>
-    <row r="109" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="24"/>
-      <c r="B109" s="11" t="s">
-        <v>108</v>
-      </c>
+      <c r="B109" s="14"/>
       <c r="C109" s="15"/>
-      <c r="D109" s="23"/>
-    </row>
-    <row r="110" ht="295" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D109" s="16" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="110" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="24"/>
-      <c r="B110" s="11"/>
+      <c r="B110" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="C110" s="15"/>
-      <c r="D110" s="10"/>
+      <c r="D110" s="23"/>
     </row>
     <row r="111" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="24"/>
-      <c r="B111" s="11" t="s">
-        <v>109</v>
+      <c r="B111" s="14" t="s">
+        <v>111</v>
       </c>
       <c r="C111" s="15"/>
       <c r="D111" s="23"/>
     </row>
-    <row r="112" ht="134" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="24"/>
-      <c r="B112" s="11"/>
+      <c r="B112" s="11" t="s">
+        <v>112</v>
+      </c>
       <c r="C112" s="15"/>
       <c r="D112" s="10"/>
     </row>
-    <row r="113" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" ht="65" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="24"/>
-      <c r="B113" s="11" t="s">
-        <v>110</v>
-      </c>
+      <c r="B113" s="11"/>
       <c r="C113" s="15"/>
-      <c r="D113" s="23"/>
-    </row>
-    <row r="114" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D113" s="10"/>
+    </row>
+    <row r="114" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="24"/>
-      <c r="B114" s="14"/>
+      <c r="B114" s="11" t="s">
+        <v>113</v>
+      </c>
       <c r="C114" s="15"/>
-      <c r="D114" s="16" t="s">
+      <c r="D114" s="23"/>
+    </row>
+    <row r="115" ht="295" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="24"/>
+      <c r="B115" s="11"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="10"/>
+    </row>
+    <row r="116" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="24"/>
+      <c r="B116" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="C116" s="15"/>
+      <c r="D116" s="23"/>
+    </row>
+    <row r="117" ht="134" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="24"/>
+      <c r="B117" s="11"/>
+      <c r="C117" s="15"/>
+      <c r="D117" s="10"/>
+    </row>
+    <row r="118" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="24"/>
+      <c r="B118" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C118" s="15"/>
+      <c r="D118" s="23"/>
+    </row>
+    <row r="119" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="24"/>
+      <c r="B119" s="14"/>
+      <c r="C119" s="15"/>
+      <c r="D119" s="16" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="115" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A115" s="26"/>
-      <c r="B115" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C115" s="27"/>
-      <c r="D115" s="10"/>
-    </row>
-    <row r="116" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" s="26"/>
-      <c r="B116" s="11"/>
-      <c r="C116" s="27"/>
-      <c r="D116" s="10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="117" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A117" s="26"/>
-      <c r="B117" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="C117" s="27"/>
-      <c r="D117" s="10"/>
-    </row>
-    <row r="118" ht="43.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" s="26"/>
-      <c r="B118" s="11"/>
-      <c r="C118" s="27"/>
-      <c r="D118" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="119" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A119" s="26"/>
-      <c r="B119" s="11"/>
-      <c r="C119" s="27"/>
-      <c r="D119" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="120" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="26"/>
       <c r="B120" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C120" s="27"/>
       <c r="D120" s="10"/>
     </row>
-    <row r="121" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="26"/>
-      <c r="B121" s="11" t="s">
-        <v>115</v>
-      </c>
+      <c r="B121" s="11"/>
       <c r="C121" s="27"/>
-      <c r="D121" s="10"/>
-    </row>
-    <row r="122" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D121" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="122" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="26"/>
-      <c r="B122" s="14"/>
+      <c r="B122" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="C122" s="27"/>
-      <c r="D122" s="16" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="123" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D122" s="10"/>
+    </row>
+    <row r="123" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="26"/>
-      <c r="B123" s="14"/>
+      <c r="B123" s="2" t="s">
+        <v>119</v>
+      </c>
       <c r="C123" s="27"/>
-      <c r="D123" s="16" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="124" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D123" s="10"/>
+    </row>
+    <row r="124" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="26"/>
-      <c r="B124" s="14"/>
+      <c r="B124" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="C124" s="27"/>
-      <c r="D124" s="28" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="125" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D124" s="10"/>
+    </row>
+    <row r="125" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="26"/>
-      <c r="B125" s="12" t="s">
-        <v>119</v>
+      <c r="B125" s="2" t="s">
+        <v>121</v>
       </c>
       <c r="C125" s="27"/>
-      <c r="D125" s="23"/>
+      <c r="D125" s="10"/>
     </row>
     <row r="126" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="26"/>
-      <c r="B126" s="12"/>
+      <c r="B126" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="C126" s="27"/>
       <c r="D126" s="10"/>
     </row>
     <row r="127" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="26"/>
-      <c r="B127" s="14" t="s">
-        <v>120</v>
+      <c r="B127" s="11" t="s">
+        <v>123</v>
       </c>
       <c r="C127" s="27"/>
-      <c r="D127" s="29"/>
-    </row>
-    <row r="128" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D127" s="10"/>
+    </row>
+    <row r="128" ht="43.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="26"/>
-      <c r="B128" s="12" t="s">
-        <v>121</v>
-      </c>
+      <c r="B128" s="11"/>
       <c r="C128" s="27"/>
-      <c r="D128" s="23"/>
+      <c r="D128" s="10" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="129" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="26"/>
-      <c r="B129" s="12"/>
+      <c r="B129" s="11"/>
       <c r="C129" s="27"/>
-      <c r="D129" s="14" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="130" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D129" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="130" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="26"/>
-      <c r="B130" s="12"/>
+      <c r="B130" s="11" t="s">
+        <v>124</v>
+      </c>
       <c r="C130" s="27"/>
-      <c r="D130" s="14" t="s">
-        <v>123</v>
-      </c>
+      <c r="D130" s="10"/>
     </row>
     <row r="131" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="26"/>
-      <c r="B131" s="12"/>
+      <c r="B131" s="11" t="s">
+        <v>125</v>
+      </c>
       <c r="C131" s="27"/>
-      <c r="D131" s="14" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="132" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D131" s="10"/>
+    </row>
+    <row r="132" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="26"/>
-      <c r="B132" s="12"/>
+      <c r="B132" s="14"/>
       <c r="C132" s="27"/>
-      <c r="D132" s="30" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="133" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D132" s="16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="133" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="26"/>
-      <c r="B133" s="12"/>
+      <c r="B133" s="14"/>
       <c r="C133" s="27"/>
-      <c r="D133" s="30" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="134" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D133" s="16" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="134" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="26"/>
-      <c r="B134" s="12"/>
+      <c r="B134" s="14"/>
       <c r="C134" s="27"/>
-      <c r="D134" s="30" t="s">
-        <v>123</v>
+      <c r="D134" s="28" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="135" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="26"/>
-      <c r="B135" s="12"/>
+      <c r="B135" s="12" t="s">
+        <v>129</v>
+      </c>
       <c r="C135" s="27"/>
-      <c r="D135" s="30" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="136" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D135" s="23"/>
+    </row>
+    <row r="136" ht="119" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="26"/>
-      <c r="B136" s="11" t="s">
-        <v>127</v>
-      </c>
+      <c r="B136" s="12"/>
       <c r="C136" s="27"/>
-      <c r="D136" s="23"/>
-    </row>
-    <row r="137" ht="153" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D136" s="10"/>
+    </row>
+    <row r="137" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="26"/>
-      <c r="B137" s="11"/>
+      <c r="B137" s="14" t="s">
+        <v>130</v>
+      </c>
       <c r="C137" s="27"/>
-      <c r="D137" s="10"/>
-    </row>
-    <row r="138" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D137" s="29"/>
+    </row>
+    <row r="138" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="26"/>
-      <c r="B138" s="11" t="s">
-        <v>128</v>
+      <c r="B138" s="12" t="s">
+        <v>131</v>
       </c>
       <c r="C138" s="27"/>
-      <c r="D138" s="31"/>
-    </row>
-    <row r="139" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D138" s="23"/>
+    </row>
+    <row r="139" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="26"/>
-      <c r="B139" s="11"/>
+      <c r="B139" s="12"/>
       <c r="C139" s="27"/>
-      <c r="D139" s="23" t="s">
-        <v>129</v>
+      <c r="D139" s="14" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="140" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="26"/>
-      <c r="B140" s="12" t="s">
-        <v>130</v>
-      </c>
+      <c r="B140" s="12"/>
       <c r="C140" s="27"/>
-      <c r="D140" s="31"/>
-    </row>
-    <row r="141" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D140" s="14" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="141" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="26"/>
       <c r="B141" s="12"/>
       <c r="C141" s="27"/>
-      <c r="D141" s="23" t="s">
-        <v>131</v>
+      <c r="D141" s="14" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="142" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="26"/>
       <c r="B142" s="12"/>
       <c r="C142" s="27"/>
-      <c r="D142" s="23" t="s">
-        <v>132</v>
+      <c r="D142" s="30" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="143" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="26"/>
-      <c r="B143" s="11" t="s">
+      <c r="B143" s="12"/>
+      <c r="C143" s="27"/>
+      <c r="D143" s="30" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="144" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A144" s="26"/>
+      <c r="B144" s="12"/>
+      <c r="C144" s="27"/>
+      <c r="D144" s="30" t="s">
         <v>133</v>
       </c>
-      <c r="C143" s="27"/>
-      <c r="D143" s="32"/>
-    </row>
-    <row r="144" ht="306" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A144" s="26"/>
-      <c r="B144" s="11"/>
-      <c r="C144" s="27"/>
-      <c r="D144" s="29" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="145" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="145" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="26"/>
-      <c r="B145" s="12" t="s">
-        <v>135</v>
-      </c>
+      <c r="B145" s="12"/>
       <c r="C145" s="27"/>
-      <c r="D145" s="33"/>
-    </row>
-    <row r="146" ht="367" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D145" s="30" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="146" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="26"/>
-      <c r="B146" s="12"/>
+      <c r="B146" s="11" t="s">
+        <v>137</v>
+      </c>
       <c r="C146" s="27"/>
-      <c r="D146" s="10"/>
-    </row>
-    <row r="147" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D146" s="23"/>
+    </row>
+    <row r="147" ht="153" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="26"/>
-      <c r="B147" s="11" t="s">
-        <v>136</v>
-      </c>
+      <c r="B147" s="11"/>
       <c r="C147" s="27"/>
-      <c r="D147" s="29"/>
+      <c r="D147" s="10"/>
     </row>
     <row r="148" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="26"/>
-      <c r="B148" s="11"/>
+      <c r="B148" s="11" t="s">
+        <v>138</v>
+      </c>
       <c r="C148" s="27"/>
-      <c r="D148" s="29" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="149" ht="51" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D148" s="31"/>
+    </row>
+    <row r="149" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="26"/>
       <c r="B149" s="11"/>
       <c r="C149" s="27"/>
-      <c r="D149" s="14" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="150" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D149" s="23" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="150" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="26"/>
-      <c r="B150" s="14" t="s">
-        <v>139</v>
+      <c r="B150" s="12" t="s">
+        <v>140</v>
       </c>
       <c r="C150" s="27"/>
-      <c r="D150" s="29"/>
-    </row>
-    <row r="151" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D150" s="31"/>
+    </row>
+    <row r="151" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="26"/>
-      <c r="B151" s="14"/>
+      <c r="B151" s="12"/>
       <c r="C151" s="27"/>
-      <c r="D151" s="28" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="152" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D151" s="23" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="152" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="26"/>
-      <c r="B152" s="12" t="s">
-        <v>141</v>
-      </c>
+      <c r="B152" s="12"/>
       <c r="C152" s="27"/>
-      <c r="D152" s="23"/>
+      <c r="D152" s="23" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="153" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="26"/>
-      <c r="B153" s="12"/>
+      <c r="B153" s="11" t="s">
+        <v>143</v>
+      </c>
       <c r="C153" s="27"/>
-      <c r="D153" s="23" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="154" ht="229" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D153" s="32"/>
+    </row>
+    <row r="154" ht="306" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="26"/>
-      <c r="B154" s="12"/>
+      <c r="B154" s="11"/>
       <c r="C154" s="27"/>
-      <c r="D154" s="10"/>
-    </row>
-    <row r="155" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D154" s="29" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="155" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="26"/>
-      <c r="B155" s="14" t="s">
-        <v>143</v>
+      <c r="B155" s="12" t="s">
+        <v>145</v>
       </c>
       <c r="C155" s="27"/>
-      <c r="D155" s="14"/>
-    </row>
-    <row r="156" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D155" s="33"/>
+    </row>
+    <row r="156" ht="367" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="26"/>
-      <c r="B156" s="12" t="s">
-        <v>144</v>
-      </c>
+      <c r="B156" s="12"/>
       <c r="C156" s="27"/>
-      <c r="D156" s="14"/>
+      <c r="D156" s="10"/>
     </row>
     <row r="157" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="26"/>
-      <c r="B157" s="12"/>
+      <c r="B157" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C157" s="27"/>
-      <c r="D157" s="14" t="s">
-        <v>145</v>
-      </c>
+      <c r="D157" s="29"/>
     </row>
     <row r="158" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="26"/>
-      <c r="B158" s="12"/>
+      <c r="B158" s="11"/>
       <c r="C158" s="27"/>
-      <c r="D158" s="14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="159" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D158" s="29" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="159" ht="51" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="26"/>
-      <c r="B159" s="12"/>
+      <c r="B159" s="11"/>
       <c r="C159" s="27"/>
-      <c r="D159" s="34" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="160" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D159" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="160" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="26"/>
-      <c r="B160" s="12"/>
+      <c r="B160" s="14" t="s">
+        <v>149</v>
+      </c>
       <c r="C160" s="27"/>
-      <c r="D160" s="14" t="s">
-        <v>147</v>
-      </c>
+      <c r="D160" s="29"/>
     </row>
     <row r="161" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="26"/>
       <c r="B161" s="14"/>
       <c r="C161" s="27"/>
       <c r="D161" s="28" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="162" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="26"/>
       <c r="B162" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C162" s="27"/>
-      <c r="D162" s="23" t="s">
-        <v>150</v>
-      </c>
+      <c r="D162" s="23"/>
     </row>
     <row r="163" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="26"/>
       <c r="B163" s="12"/>
       <c r="C163" s="27"/>
       <c r="D163" s="23" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="164" ht="222" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="164" ht="229" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="26"/>
-      <c r="B164" s="11" t="s">
-        <v>149</v>
-      </c>
+      <c r="B164" s="12"/>
       <c r="C164" s="27"/>
       <c r="D164" s="10"/>
     </row>
     <row r="165" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="26"/>
       <c r="B165" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C165" s="27"/>
       <c r="D165" s="14"/>
@@ -5908,7 +5960,7 @@
     <row r="166" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="26"/>
       <c r="B166" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C166" s="27"/>
       <c r="D166" s="14"/>
@@ -5918,7 +5970,7 @@
       <c r="B167" s="12"/>
       <c r="C167" s="27"/>
       <c r="D167" s="14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="168" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5926,7 +5978,7 @@
       <c r="B168" s="12"/>
       <c r="C168" s="27"/>
       <c r="D168" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="169" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5942,7 +5994,7 @@
       <c r="B170" s="12"/>
       <c r="C170" s="27"/>
       <c r="D170" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="171" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5950,17 +6002,17 @@
       <c r="B171" s="14"/>
       <c r="C171" s="27"/>
       <c r="D171" s="28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="172" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="26"/>
       <c r="B172" s="12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C172" s="27"/>
       <c r="D172" s="23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="173" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5968,13 +6020,13 @@
       <c r="B173" s="12"/>
       <c r="C173" s="27"/>
       <c r="D173" s="23" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="174" ht="227" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="174" ht="222" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="26"/>
       <c r="B174" s="11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C174" s="27"/>
       <c r="D174" s="10"/>
@@ -5982,7 +6034,7 @@
     <row r="175" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="26"/>
       <c r="B175" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C175" s="27"/>
       <c r="D175" s="14"/>
@@ -5990,7 +6042,7 @@
     <row r="176" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="26"/>
       <c r="B176" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C176" s="27"/>
       <c r="D176" s="14"/>
@@ -6000,7 +6052,7 @@
       <c r="B177" s="12"/>
       <c r="C177" s="27"/>
       <c r="D177" s="14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="178" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6008,7 +6060,7 @@
       <c r="B178" s="12"/>
       <c r="C178" s="27"/>
       <c r="D178" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="179" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6024,175 +6076,177 @@
       <c r="B180" s="12"/>
       <c r="C180" s="27"/>
       <c r="D180" s="14" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="181" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="181" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" s="26"/>
-      <c r="B181" s="12" t="s">
-        <v>166</v>
-      </c>
+      <c r="B181" s="14"/>
       <c r="C181" s="27"/>
-      <c r="D181" s="14"/>
+      <c r="D181" s="28" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="182" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" s="26"/>
-      <c r="B182" s="14"/>
+      <c r="B182" s="12" t="s">
+        <v>168</v>
+      </c>
       <c r="C182" s="27"/>
-      <c r="D182" s="28" t="s">
-        <v>167</v>
+      <c r="D182" s="23" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="183" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="26"/>
-      <c r="B183" s="14" t="s">
+      <c r="B183" s="12"/>
+      <c r="C183" s="27"/>
+      <c r="D183" s="23" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="184" ht="227" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A184" s="26"/>
+      <c r="B184" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C183" s="27"/>
-      <c r="D183" s="23"/>
-    </row>
-    <row r="184" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A184" s="26"/>
-      <c r="B184" s="14"/>
       <c r="C184" s="27"/>
-      <c r="D184" s="28" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="185" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D184" s="10"/>
+    </row>
+    <row r="185" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" s="26"/>
-      <c r="B185" s="12" t="s">
-        <v>170</v>
+      <c r="B185" s="14" t="s">
+        <v>171</v>
       </c>
       <c r="C185" s="27"/>
-      <c r="D185" s="35"/>
+      <c r="D185" s="14"/>
     </row>
     <row r="186" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" s="26"/>
-      <c r="B186" s="12"/>
+      <c r="B186" s="12" t="s">
+        <v>172</v>
+      </c>
       <c r="C186" s="27"/>
-      <c r="D186" s="10" t="s">
-        <v>21</v>
-      </c>
+      <c r="D186" s="14"/>
     </row>
     <row r="187" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" s="26"/>
       <c r="B187" s="12"/>
       <c r="C187" s="27"/>
-      <c r="D187" s="10" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="188" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D187" s="14" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="188" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" s="26"/>
       <c r="B188" s="12"/>
       <c r="C188" s="27"/>
-      <c r="D188" s="23" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="189" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D188" s="14" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="189" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" s="26"/>
-      <c r="B189" s="14"/>
+      <c r="B189" s="12"/>
       <c r="C189" s="27"/>
-      <c r="D189" s="28" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="190" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D189" s="34" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="190" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" s="26"/>
-      <c r="B190" s="12" t="s">
-        <v>174</v>
-      </c>
+      <c r="B190" s="12"/>
       <c r="C190" s="27"/>
-      <c r="D190" s="35"/>
-    </row>
-    <row r="191" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D190" s="14" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="191" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="26"/>
-      <c r="B191" s="12"/>
+      <c r="B191" s="12" t="s">
+        <v>176</v>
+      </c>
       <c r="C191" s="27"/>
-      <c r="D191" s="10" t="s">
-        <v>21</v>
-      </c>
+      <c r="D191" s="14"/>
     </row>
     <row r="192" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="26"/>
-      <c r="B192" s="12"/>
+      <c r="B192" s="14"/>
       <c r="C192" s="27"/>
-      <c r="D192" s="10" t="s">
-        <v>175</v>
+      <c r="D192" s="28" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="193" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" s="26"/>
-      <c r="B193" s="12"/>
+      <c r="B193" s="14" t="s">
+        <v>178</v>
+      </c>
       <c r="C193" s="27"/>
-      <c r="D193" s="23" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="194" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D193" s="23"/>
+    </row>
+    <row r="194" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="26"/>
       <c r="B194" s="14"/>
       <c r="C194" s="27"/>
-      <c r="D194" s="36" t="s">
-        <v>177</v>
+      <c r="D194" s="28" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="195" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" s="26"/>
       <c r="B195" s="12" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C195" s="27"/>
-      <c r="D195" s="29"/>
+      <c r="D195" s="35"/>
     </row>
     <row r="196" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" s="26"/>
       <c r="B196" s="12"/>
       <c r="C196" s="27"/>
-      <c r="D196" s="14" t="s">
-        <v>179</v>
+      <c r="D196" s="10" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="197" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" s="26"/>
       <c r="B197" s="12"/>
       <c r="C197" s="27"/>
-      <c r="D197" s="14" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="198" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D197" s="10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="198" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" s="26"/>
       <c r="B198" s="12"/>
       <c r="C198" s="27"/>
-      <c r="D198" s="14" t="s">
-        <v>181</v>
+      <c r="D198" s="23" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="199" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" s="26"/>
-      <c r="B199" s="12"/>
+      <c r="B199" s="14"/>
       <c r="C199" s="27"/>
-      <c r="D199" s="10" t="s">
-        <v>182</v>
+      <c r="D199" s="28" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="200" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" s="26"/>
-      <c r="B200" s="12"/>
+      <c r="B200" s="12" t="s">
+        <v>184</v>
+      </c>
       <c r="C200" s="27"/>
-      <c r="D200" s="10" t="s">
-        <v>183</v>
-      </c>
+      <c r="D200" s="35"/>
     </row>
     <row r="201" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" s="26"/>
       <c r="B201" s="12"/>
       <c r="C201" s="27"/>
       <c r="D201" s="10" t="s">
-        <v>184</v>
+        <v>21</v>
       </c>
     </row>
     <row r="202" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6203,35 +6257,35 @@
         <v>185</v>
       </c>
     </row>
-    <row r="203" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="203" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" s="26"/>
       <c r="B203" s="12"/>
       <c r="C203" s="27"/>
-      <c r="D203" s="10" t="s">
+      <c r="D203" s="23" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="204" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="204" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" s="26"/>
-      <c r="B204" s="12"/>
+      <c r="B204" s="14"/>
       <c r="C204" s="27"/>
-      <c r="D204" s="10" t="s">
+      <c r="D204" s="36" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="205" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" s="26"/>
-      <c r="B205" s="12"/>
+      <c r="B205" s="12" t="s">
+        <v>188</v>
+      </c>
       <c r="C205" s="27"/>
-      <c r="D205" s="10" t="s">
-        <v>188</v>
-      </c>
+      <c r="D205" s="29"/>
     </row>
     <row r="206" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" s="26"/>
       <c r="B206" s="12"/>
       <c r="C206" s="27"/>
-      <c r="D206" s="10" t="s">
+      <c r="D206" s="14" t="s">
         <v>189</v>
       </c>
     </row>
@@ -6239,7 +6293,7 @@
       <c r="A207" s="26"/>
       <c r="B207" s="12"/>
       <c r="C207" s="27"/>
-      <c r="D207" s="10" t="s">
+      <c r="D207" s="14" t="s">
         <v>190</v>
       </c>
     </row>
@@ -6247,7 +6301,7 @@
       <c r="A208" s="26"/>
       <c r="B208" s="12"/>
       <c r="C208" s="27"/>
-      <c r="D208" s="10" t="s">
+      <c r="D208" s="14" t="s">
         <v>191</v>
       </c>
     </row>
@@ -6709,334 +6763,370 @@
     </row>
     <row r="266" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" s="26"/>
-      <c r="B266" s="14"/>
+      <c r="B266" s="12"/>
       <c r="C266" s="27"/>
-      <c r="D266" s="16" t="s">
+      <c r="D266" s="10" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="267" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="267" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" s="26"/>
-      <c r="B267" s="11" t="s">
+      <c r="B267" s="12"/>
+      <c r="C267" s="27"/>
+      <c r="D267" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="C267" s="27"/>
-      <c r="D267" s="29"/>
-    </row>
-    <row r="268" ht="236" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="268" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" s="26"/>
-      <c r="B268" s="11"/>
+      <c r="B268" s="12"/>
       <c r="C268" s="27"/>
-      <c r="D268" s="10"/>
+      <c r="D268" s="10" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="269" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" s="26"/>
-      <c r="B269" s="11" t="s">
-        <v>251</v>
-      </c>
+      <c r="B269" s="12"/>
       <c r="C269" s="27"/>
-      <c r="D269" s="29"/>
-    </row>
-    <row r="270" ht="159" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D269" s="10" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="270" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" s="26"/>
-      <c r="B270" s="11"/>
+      <c r="B270" s="12"/>
       <c r="C270" s="27"/>
-      <c r="D270" s="10"/>
+      <c r="D270" s="10" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="271" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" s="26"/>
-      <c r="B271" s="11" t="s">
-        <v>252</v>
-      </c>
+      <c r="B271" s="12"/>
       <c r="C271" s="27"/>
-      <c r="D271" s="29"/>
-    </row>
-    <row r="272" ht="124" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D271" s="10" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="272" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" s="26"/>
-      <c r="B272" s="11"/>
+      <c r="B272" s="12"/>
       <c r="C272" s="27"/>
-      <c r="D272" s="10"/>
+      <c r="D272" s="10" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="273" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" s="26"/>
-      <c r="B273" s="11" t="s">
-        <v>253</v>
-      </c>
+      <c r="B273" s="12"/>
       <c r="C273" s="27"/>
-      <c r="D273" s="29"/>
-    </row>
-    <row r="274" ht="231" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D273" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="274" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" s="26"/>
-      <c r="B274" s="11"/>
+      <c r="B274" s="12"/>
       <c r="C274" s="27"/>
-      <c r="D274" s="10"/>
+      <c r="D274" s="10" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="275" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" s="26"/>
-      <c r="B275" s="12" t="s">
-        <v>254</v>
-      </c>
+      <c r="B275" s="12"/>
       <c r="C275" s="27"/>
-      <c r="D275" s="29"/>
+      <c r="D275" s="10" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="276" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" s="26"/>
-      <c r="B276" s="12"/>
+      <c r="B276" s="14"/>
       <c r="C276" s="27"/>
-      <c r="D276" s="29" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="277" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D276" s="16" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="277" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" s="26"/>
-      <c r="B277" s="12"/>
+      <c r="B277" s="11" t="s">
+        <v>260</v>
+      </c>
       <c r="C277" s="27"/>
-      <c r="D277" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="278" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D277" s="29"/>
+    </row>
+    <row r="278" ht="236" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" s="26"/>
-      <c r="B278" s="12"/>
+      <c r="B278" s="11"/>
       <c r="C278" s="27"/>
-      <c r="D278" s="10" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="279" ht="207" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D278" s="10"/>
+    </row>
+    <row r="279" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" s="26"/>
-      <c r="B279" s="12"/>
+      <c r="B279" s="11" t="s">
+        <v>261</v>
+      </c>
       <c r="C279" s="27"/>
-      <c r="D279" s="10"/>
-    </row>
-    <row r="280" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A280" s="37"/>
-      <c r="B280" s="14"/>
+      <c r="D279" s="29"/>
+    </row>
+    <row r="280" ht="159" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A280" s="26"/>
+      <c r="B280" s="11"/>
       <c r="C280" s="27"/>
       <c r="D280" s="10"/>
     </row>
-    <row r="281" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A281" s="37"/>
-      <c r="B281" s="14"/>
+    <row r="281" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A281" s="26"/>
+      <c r="B281" s="11" t="s">
+        <v>262</v>
+      </c>
       <c r="C281" s="27"/>
-      <c r="D281" s="10"/>
-    </row>
-    <row r="282" ht="75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A282" s="38" t="s">
-        <v>257</v>
-      </c>
-      <c r="B282" s="14"/>
-      <c r="C282" s="15" t="s">
+      <c r="D281" s="29"/>
+    </row>
+    <row r="282" ht="124" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A282" s="26"/>
+      <c r="B282" s="11"/>
+      <c r="C282" s="27"/>
+      <c r="D282" s="10"/>
+    </row>
+    <row r="283" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A283" s="26"/>
+      <c r="B283" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="C283" s="27"/>
+      <c r="D283" s="29"/>
+    </row>
+    <row r="284" ht="231" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A284" s="26"/>
+      <c r="B284" s="11"/>
+      <c r="C284" s="27"/>
+      <c r="D284" s="10"/>
+    </row>
+    <row r="285" ht="231" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A285" s="26"/>
+      <c r="B285" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C285" s="27"/>
+      <c r="D285" s="10"/>
+    </row>
+    <row r="286" ht="231" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A286" s="26"/>
+      <c r="B286" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C286" s="27"/>
+      <c r="D286" s="10"/>
+    </row>
+    <row r="287" ht="231" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A287" s="26"/>
+      <c r="B287" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C287" s="27"/>
+      <c r="D287" s="10"/>
+    </row>
+    <row r="288" ht="231" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A288" s="26"/>
+      <c r="B288" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C288" s="27"/>
+      <c r="D288" s="10"/>
+    </row>
+    <row r="289" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A289" s="26"/>
+      <c r="B289" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="C289" s="27"/>
+      <c r="D289" s="29"/>
+    </row>
+    <row r="290" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A290" s="26"/>
+      <c r="B290" s="12"/>
+      <c r="C290" s="27"/>
+      <c r="D290" s="29" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="291" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A291" s="26"/>
+      <c r="B291" s="12"/>
+      <c r="C291" s="27"/>
+      <c r="D291" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="292" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A292" s="26"/>
+      <c r="B292" s="12"/>
+      <c r="C292" s="27"/>
+      <c r="D292" s="10" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="293" ht="207" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A293" s="26"/>
+      <c r="B293" s="12"/>
+      <c r="C293" s="27"/>
+      <c r="D293" s="10"/>
+    </row>
+    <row r="294" ht="207" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A294" s="26"/>
+      <c r="B294" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C294" s="27"/>
+      <c r="D294" s="10"/>
+    </row>
+    <row r="295" ht="207" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A295" s="26"/>
+      <c r="B295" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C295" s="27"/>
+      <c r="D295" s="10"/>
+    </row>
+    <row r="296" ht="207" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A296" s="26"/>
+      <c r="B296" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C296" s="27"/>
+      <c r="D296" s="10"/>
+    </row>
+    <row r="297" ht="207" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A297" s="26"/>
+      <c r="B297" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C297" s="27"/>
+      <c r="D297" s="10"/>
+    </row>
+    <row r="298" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A298" s="37"/>
+      <c r="B298" s="14"/>
+      <c r="C298" s="27"/>
+      <c r="D298" s="10"/>
+    </row>
+    <row r="299" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A299" s="37"/>
+      <c r="B299" s="14"/>
+      <c r="C299" s="27"/>
+      <c r="D299" s="10"/>
+    </row>
+    <row r="300" ht="75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A300" s="38" t="s">
+        <v>275</v>
+      </c>
+      <c r="B300" s="14"/>
+      <c r="C300" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D282" s="10"/>
-    </row>
-    <row r="283" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A283" s="38"/>
-      <c r="B283" s="14"/>
-      <c r="C283" s="15"/>
-      <c r="D283" s="10"/>
-    </row>
-    <row r="284" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A284" s="38"/>
-      <c r="B284" s="14"/>
-      <c r="C284" s="15" t="s">
-        <v>258</v>
-      </c>
-      <c r="D284" s="10"/>
-    </row>
-    <row r="285" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A285" s="38"/>
-      <c r="B285" s="14"/>
-      <c r="C285" s="15"/>
-      <c r="D285" s="10"/>
-    </row>
-    <row r="286" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A286" s="38"/>
-      <c r="B286" s="14"/>
-      <c r="C286" s="15"/>
-      <c r="D286" s="10"/>
-    </row>
-    <row r="287" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A287" s="38"/>
-      <c r="B287" s="14"/>
-      <c r="C287" s="15"/>
-      <c r="D287" s="10"/>
-    </row>
-    <row r="288" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A288" s="38"/>
-      <c r="B288" s="14"/>
-      <c r="C288" s="15"/>
-      <c r="D288" s="10"/>
-    </row>
-    <row r="289" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A289" s="38"/>
-      <c r="B289" s="14"/>
-      <c r="C289" s="15"/>
-      <c r="D289" s="10"/>
-    </row>
-    <row r="290" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A290" s="38"/>
-      <c r="B290" s="14"/>
-      <c r="C290" s="15"/>
-      <c r="D290" s="10"/>
-    </row>
-    <row r="291" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A291" s="38"/>
-      <c r="B291" s="14"/>
-      <c r="C291" s="15"/>
-      <c r="D291" s="10"/>
-    </row>
-    <row r="292" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A292" s="38"/>
-      <c r="B292" s="14"/>
-      <c r="C292" s="15"/>
-      <c r="D292" s="10"/>
-    </row>
-    <row r="293" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A293" s="38"/>
-      <c r="B293" s="14"/>
-      <c r="C293" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D293" s="10"/>
-    </row>
-    <row r="294" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A294" s="38"/>
-      <c r="B294" s="14"/>
-      <c r="C294" s="15"/>
-      <c r="D294" s="10"/>
-    </row>
-    <row r="295" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A295" s="38"/>
-      <c r="B295" s="14"/>
-      <c r="C295" s="15"/>
-      <c r="D295" s="10"/>
-    </row>
-    <row r="296" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A296" s="38"/>
-      <c r="B296" s="14"/>
-      <c r="C296" s="15"/>
-      <c r="D296" s="10"/>
-    </row>
-    <row r="297" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A297" s="38"/>
-      <c r="B297" s="14"/>
-      <c r="C297" s="15"/>
-      <c r="D297" s="10"/>
-    </row>
-    <row r="298" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A298" s="39" t="s">
-        <v>259</v>
-      </c>
-      <c r="B298" s="14"/>
-      <c r="C298" s="40"/>
-      <c r="D298" s="10"/>
-    </row>
-    <row r="299" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A299" s="39"/>
-      <c r="B299" s="14"/>
-      <c r="C299" s="40"/>
-      <c r="D299" s="10"/>
-    </row>
-    <row r="300" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A300" s="39"/>
-      <c r="B300" s="14"/>
-      <c r="C300" s="40"/>
       <c r="D300" s="10"/>
     </row>
     <row r="301" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A301" s="39"/>
+      <c r="A301" s="38"/>
       <c r="B301" s="14"/>
-      <c r="C301" s="40"/>
+      <c r="C301" s="15"/>
       <c r="D301" s="10"/>
     </row>
     <row r="302" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A302" s="39"/>
+      <c r="A302" s="38"/>
       <c r="B302" s="14"/>
-      <c r="C302" s="40"/>
+      <c r="C302" s="15" t="s">
+        <v>276</v>
+      </c>
       <c r="D302" s="10"/>
     </row>
-    <row r="303" ht="63.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A303" s="39"/>
+    <row r="303" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A303" s="38"/>
       <c r="B303" s="14"/>
-      <c r="C303" s="40"/>
+      <c r="C303" s="15"/>
       <c r="D303" s="10"/>
     </row>
     <row r="304" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A304" s="39"/>
+      <c r="A304" s="38"/>
       <c r="B304" s="14"/>
-      <c r="C304" s="40"/>
+      <c r="C304" s="15"/>
       <c r="D304" s="10"/>
     </row>
     <row r="305" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A305" s="39"/>
+      <c r="A305" s="38"/>
       <c r="B305" s="14"/>
-      <c r="C305" s="40"/>
+      <c r="C305" s="15"/>
       <c r="D305" s="10"/>
     </row>
     <row r="306" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A306" s="39"/>
+      <c r="A306" s="38"/>
       <c r="B306" s="14"/>
-      <c r="C306" s="40"/>
+      <c r="C306" s="15"/>
       <c r="D306" s="10"/>
     </row>
     <row r="307" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A307" s="39"/>
+      <c r="A307" s="38"/>
       <c r="B307" s="14"/>
-      <c r="C307" s="40"/>
+      <c r="C307" s="15"/>
       <c r="D307" s="10"/>
     </row>
     <row r="308" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A308" s="39"/>
+      <c r="A308" s="38"/>
       <c r="B308" s="14"/>
-      <c r="C308" s="40"/>
+      <c r="C308" s="15"/>
       <c r="D308" s="10"/>
     </row>
-    <row r="309" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A309" s="39"/>
+    <row r="309" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A309" s="38"/>
       <c r="B309" s="14"/>
-      <c r="C309" s="40"/>
+      <c r="C309" s="15"/>
       <c r="D309" s="10"/>
     </row>
     <row r="310" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A310" s="39"/>
+      <c r="A310" s="38"/>
       <c r="B310" s="14"/>
-      <c r="C310" s="40"/>
+      <c r="C310" s="15"/>
       <c r="D310" s="10"/>
     </row>
     <row r="311" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A311" s="39"/>
+      <c r="A311" s="38"/>
       <c r="B311" s="14"/>
-      <c r="C311" s="40"/>
+      <c r="C311" s="15" t="s">
+        <v>77</v>
+      </c>
       <c r="D311" s="10"/>
     </row>
     <row r="312" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A312" s="39"/>
+      <c r="A312" s="38"/>
       <c r="B312" s="14"/>
-      <c r="C312" s="40"/>
+      <c r="C312" s="15"/>
       <c r="D312" s="10"/>
     </row>
     <row r="313" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A313" s="39"/>
+      <c r="A313" s="38"/>
       <c r="B313" s="14"/>
-      <c r="C313" s="40"/>
+      <c r="C313" s="15"/>
       <c r="D313" s="10"/>
     </row>
     <row r="314" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A314" s="39"/>
+      <c r="A314" s="38"/>
       <c r="B314" s="14"/>
-      <c r="C314" s="40"/>
+      <c r="C314" s="15"/>
       <c r="D314" s="10"/>
     </row>
     <row r="315" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A315" s="39"/>
+      <c r="A315" s="38"/>
       <c r="B315" s="14"/>
-      <c r="C315" s="40"/>
+      <c r="C315" s="15"/>
       <c r="D315" s="10"/>
     </row>
     <row r="316" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A316" s="39"/>
+      <c r="A316" s="39" t="s">
+        <v>277</v>
+      </c>
       <c r="B316" s="14"/>
       <c r="C316" s="40"/>
       <c r="D316" s="10"/>
@@ -7047,7 +7137,7 @@
       <c r="C317" s="40"/>
       <c r="D317" s="10"/>
     </row>
-    <row r="318" ht="216.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="318" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" s="39"/>
       <c r="B318" s="14"/>
       <c r="C318" s="40"/>
@@ -7056,16 +7146,16 @@
     <row r="319" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" s="39"/>
       <c r="B319" s="14"/>
-      <c r="C319" s="2"/>
+      <c r="C319" s="40"/>
       <c r="D319" s="10"/>
     </row>
-    <row r="320" ht="128.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="320" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" s="39"/>
       <c r="B320" s="14"/>
       <c r="C320" s="40"/>
       <c r="D320" s="10"/>
     </row>
-    <row r="321" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="321" ht="63.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" s="39"/>
       <c r="B321" s="14"/>
       <c r="C321" s="40"/>
@@ -7077,7 +7167,7 @@
       <c r="C322" s="40"/>
       <c r="D322" s="10"/>
     </row>
-    <row r="323" ht="16.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="323" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" s="39"/>
       <c r="B323" s="14"/>
       <c r="C323" s="40"/>
@@ -7095,7 +7185,7 @@
       <c r="C325" s="40"/>
       <c r="D325" s="10"/>
     </row>
-    <row r="326" ht="60" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="326" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" s="39"/>
       <c r="B326" s="14"/>
       <c r="C326" s="40"/>
@@ -7155,7 +7245,7 @@
       <c r="C335" s="40"/>
       <c r="D335" s="10"/>
     </row>
-    <row r="336" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="336" ht="216.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" s="39"/>
       <c r="B336" s="14"/>
       <c r="C336" s="40"/>
@@ -7164,10 +7254,10 @@
     <row r="337" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" s="39"/>
       <c r="B337" s="14"/>
-      <c r="C337" s="40"/>
+      <c r="C337" s="2"/>
       <c r="D337" s="10"/>
     </row>
-    <row r="338" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="338" ht="128.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" s="39"/>
       <c r="B338" s="14"/>
       <c r="C338" s="40"/>
@@ -7179,297 +7269,405 @@
       <c r="C339" s="40"/>
       <c r="D339" s="10"/>
     </row>
-    <row r="340" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A340" s="41" t="s">
-        <v>260</v>
-      </c>
+    <row r="340" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A340" s="39"/>
       <c r="B340" s="14"/>
-      <c r="C340" s="7" t="s">
-        <v>72</v>
-      </c>
+      <c r="C340" s="40"/>
       <c r="D340" s="10"/>
     </row>
-    <row r="341" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A341" s="41"/>
+    <row r="341" ht="16.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A341" s="39"/>
       <c r="B341" s="14"/>
-      <c r="C341" s="7"/>
+      <c r="C341" s="40"/>
       <c r="D341" s="10"/>
     </row>
     <row r="342" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A342" s="41"/>
+      <c r="A342" s="39"/>
       <c r="B342" s="14"/>
-      <c r="C342" s="7"/>
+      <c r="C342" s="40"/>
       <c r="D342" s="10"/>
     </row>
     <row r="343" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A343" s="41"/>
+      <c r="A343" s="39"/>
       <c r="B343" s="14"/>
-      <c r="C343" s="7"/>
+      <c r="C343" s="40"/>
       <c r="D343" s="10"/>
     </row>
-    <row r="344" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A344" s="41"/>
+    <row r="344" ht="60" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A344" s="39"/>
       <c r="B344" s="14"/>
-      <c r="C344" s="7"/>
+      <c r="C344" s="40"/>
       <c r="D344" s="10"/>
     </row>
     <row r="345" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A345" s="41"/>
+      <c r="A345" s="39"/>
       <c r="B345" s="14"/>
-      <c r="C345" s="7"/>
+      <c r="C345" s="40"/>
       <c r="D345" s="10"/>
     </row>
     <row r="346" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A346" s="41"/>
+      <c r="A346" s="39"/>
       <c r="B346" s="14"/>
-      <c r="C346" s="7"/>
+      <c r="C346" s="40"/>
       <c r="D346" s="10"/>
     </row>
     <row r="347" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A347" s="41"/>
+      <c r="A347" s="39"/>
       <c r="B347" s="14"/>
-      <c r="C347" s="7"/>
+      <c r="C347" s="40"/>
       <c r="D347" s="10"/>
     </row>
-    <row r="348" ht="105" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A348" s="41"/>
+    <row r="348" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A348" s="39"/>
       <c r="B348" s="14"/>
-      <c r="C348" s="7" t="s">
-        <v>72</v>
-      </c>
+      <c r="C348" s="40"/>
       <c r="D348" s="10"/>
     </row>
     <row r="349" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A349" s="41"/>
+      <c r="A349" s="39"/>
       <c r="B349" s="14"/>
-      <c r="C349" s="7"/>
+      <c r="C349" s="40"/>
       <c r="D349" s="10"/>
     </row>
     <row r="350" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A350" s="39" t="s">
-        <v>261</v>
-      </c>
+      <c r="A350" s="39"/>
       <c r="B350" s="14"/>
-      <c r="C350" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="C350" s="40"/>
       <c r="D350" s="10"/>
     </row>
-    <row r="351" ht="34.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="351" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" s="39"/>
       <c r="B351" s="14"/>
-      <c r="C351" s="15"/>
+      <c r="C351" s="40"/>
       <c r="D351" s="10"/>
     </row>
     <row r="352" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" s="39"/>
       <c r="B352" s="14"/>
-      <c r="C352" s="15"/>
+      <c r="C352" s="40"/>
       <c r="D352" s="10"/>
     </row>
     <row r="353" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" s="39"/>
       <c r="B353" s="14"/>
-      <c r="C353" s="15"/>
+      <c r="C353" s="40"/>
       <c r="D353" s="10"/>
     </row>
     <row r="354" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" s="39"/>
       <c r="B354" s="14"/>
-      <c r="C354" s="15"/>
+      <c r="C354" s="40"/>
       <c r="D354" s="10"/>
     </row>
     <row r="355" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" s="39"/>
       <c r="B355" s="14"/>
-      <c r="C355" s="15"/>
+      <c r="C355" s="40"/>
       <c r="D355" s="10"/>
     </row>
-    <row r="356" ht="162.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A356" s="42" t="s">
-        <v>262</v>
-      </c>
+    <row r="356" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A356" s="39"/>
       <c r="B356" s="14"/>
-      <c r="C356" s="15" t="s">
-        <v>263</v>
-      </c>
+      <c r="C356" s="40"/>
       <c r="D356" s="10"/>
     </row>
     <row r="357" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A357" s="42"/>
+      <c r="A357" s="39"/>
       <c r="B357" s="14"/>
-      <c r="C357" s="15"/>
+      <c r="C357" s="40"/>
       <c r="D357" s="10"/>
     </row>
-    <row r="358" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A358" s="42"/>
+    <row r="358" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A358" s="41" t="s">
+        <v>278</v>
+      </c>
       <c r="B358" s="14"/>
-      <c r="C358" s="15"/>
+      <c r="C358" s="7" t="s">
+        <v>77</v>
+      </c>
       <c r="D358" s="10"/>
     </row>
     <row r="359" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A359" s="42"/>
+      <c r="A359" s="41"/>
       <c r="B359" s="14"/>
-      <c r="C359" s="15"/>
+      <c r="C359" s="7"/>
       <c r="D359" s="10"/>
     </row>
-    <row r="360" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A360" s="42"/>
+    <row r="360" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A360" s="41"/>
       <c r="B360" s="14"/>
-      <c r="C360" s="15"/>
+      <c r="C360" s="7"/>
       <c r="D360" s="10"/>
     </row>
     <row r="361" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A361" s="42"/>
+      <c r="A361" s="41"/>
       <c r="B361" s="14"/>
-      <c r="C361" s="15"/>
+      <c r="C361" s="7"/>
       <c r="D361" s="10"/>
     </row>
     <row r="362" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A362" s="42"/>
+      <c r="A362" s="41"/>
       <c r="B362" s="14"/>
-      <c r="C362" s="15"/>
+      <c r="C362" s="7"/>
       <c r="D362" s="10"/>
     </row>
-    <row r="363" ht="35.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A363" s="42" t="s">
-        <v>264</v>
-      </c>
+    <row r="363" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A363" s="41"/>
       <c r="B363" s="14"/>
-      <c r="C363" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="C363" s="7"/>
       <c r="D363" s="10"/>
     </row>
     <row r="364" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A364" s="42"/>
+      <c r="A364" s="41"/>
       <c r="B364" s="14"/>
-      <c r="C364" s="15"/>
+      <c r="C364" s="7"/>
       <c r="D364" s="10"/>
     </row>
     <row r="365" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A365" s="42"/>
+      <c r="A365" s="41"/>
       <c r="B365" s="14"/>
-      <c r="C365" s="15"/>
+      <c r="C365" s="7"/>
       <c r="D365" s="10"/>
     </row>
-    <row r="366" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A366" s="42"/>
+    <row r="366" ht="105" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A366" s="41"/>
       <c r="B366" s="14"/>
-      <c r="C366" s="15"/>
+      <c r="C366" s="7" t="s">
+        <v>77</v>
+      </c>
       <c r="D366" s="10"/>
     </row>
-    <row r="367" ht="48.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A367" s="43" t="s">
-        <v>265</v>
-      </c>
+    <row r="367" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A367" s="41"/>
       <c r="B367" s="14"/>
-      <c r="C367" s="15" t="s">
-        <v>266</v>
-      </c>
+      <c r="C367" s="7"/>
       <c r="D367" s="10"/>
     </row>
     <row r="368" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A368" s="43"/>
+      <c r="A368" s="39" t="s">
+        <v>279</v>
+      </c>
       <c r="B368" s="14"/>
-      <c r="C368" s="15"/>
+      <c r="C368" s="15" t="s">
+        <v>77</v>
+      </c>
       <c r="D368" s="10"/>
     </row>
-    <row r="369" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A369" s="43"/>
+    <row r="369" ht="34.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A369" s="39"/>
       <c r="B369" s="14"/>
       <c r="C369" s="15"/>
       <c r="D369" s="10"/>
     </row>
     <row r="370" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A370" s="43"/>
+      <c r="A370" s="39"/>
       <c r="B370" s="14"/>
       <c r="C370" s="15"/>
       <c r="D370" s="10"/>
     </row>
     <row r="371" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A371" s="43"/>
+      <c r="A371" s="39"/>
       <c r="B371" s="14"/>
       <c r="C371" s="15"/>
       <c r="D371" s="10"/>
     </row>
     <row r="372" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A372" s="43"/>
+      <c r="A372" s="39"/>
       <c r="B372" s="14"/>
       <c r="C372" s="15"/>
       <c r="D372" s="10"/>
     </row>
     <row r="373" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A373" s="43"/>
+      <c r="A373" s="39"/>
       <c r="B373" s="14"/>
       <c r="C373" s="15"/>
       <c r="D373" s="10"/>
     </row>
-    <row r="374" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A374" s="43"/>
-      <c r="B374" s="44"/>
-      <c r="C374" s="15"/>
-      <c r="D374" s="45"/>
-    </row>
-    <row r="375" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A375" s="43"/>
-      <c r="B375" s="46"/>
+    <row r="374" ht="162.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A374" s="42" t="s">
+        <v>280</v>
+      </c>
+      <c r="B374" s="14"/>
+      <c r="C374" s="15" t="s">
+        <v>281</v>
+      </c>
+      <c r="D374" s="10"/>
+    </row>
+    <row r="375" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A375" s="42"/>
+      <c r="B375" s="14"/>
       <c r="C375" s="15"/>
-      <c r="D375" s="45"/>
-    </row>
-    <row r="376" ht="52.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A376" s="43"/>
-      <c r="B376" s="47"/>
-      <c r="C376" s="15" t="s">
-        <v>266</v>
-      </c>
-      <c r="D376" s="2"/>
-    </row>
-    <row r="377" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A377" s="43"/>
-      <c r="B377" s="44"/>
+      <c r="D375" s="10"/>
+    </row>
+    <row r="376" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A376" s="42"/>
+      <c r="B376" s="14"/>
+      <c r="C376" s="15"/>
+      <c r="D376" s="10"/>
+    </row>
+    <row r="377" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A377" s="42"/>
+      <c r="B377" s="14"/>
       <c r="C377" s="15"/>
-      <c r="D377" s="2"/>
-    </row>
-    <row r="378" ht="38.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A378" s="43"/>
-      <c r="B378" s="46"/>
+      <c r="D377" s="10"/>
+    </row>
+    <row r="378" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A378" s="42"/>
+      <c r="B378" s="14"/>
       <c r="C378" s="15"/>
-      <c r="D378" s="2"/>
-    </row>
-    <row r="379" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A379" s="39" t="s">
-        <v>267</v>
-      </c>
-      <c r="B379" s="47"/>
-      <c r="C379" s="15" t="s">
+      <c r="D378" s="10"/>
+    </row>
+    <row r="379" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A379" s="42"/>
+      <c r="B379" s="14"/>
+      <c r="C379" s="15"/>
+      <c r="D379" s="10"/>
+    </row>
+    <row r="380" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A380" s="42"/>
+      <c r="B380" s="14"/>
+      <c r="C380" s="15"/>
+      <c r="D380" s="10"/>
+    </row>
+    <row r="381" ht="35.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A381" s="42" t="s">
+        <v>282</v>
+      </c>
+      <c r="B381" s="14"/>
+      <c r="C381" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D381" s="10"/>
+    </row>
+    <row r="382" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A382" s="42"/>
+      <c r="B382" s="14"/>
+      <c r="C382" s="15"/>
+      <c r="D382" s="10"/>
+    </row>
+    <row r="383" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A383" s="42"/>
+      <c r="B383" s="14"/>
+      <c r="C383" s="15"/>
+      <c r="D383" s="10"/>
+    </row>
+    <row r="384" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A384" s="42"/>
+      <c r="B384" s="14"/>
+      <c r="C384" s="15"/>
+      <c r="D384" s="10"/>
+    </row>
+    <row r="385" ht="48.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A385" s="43" t="s">
+        <v>283</v>
+      </c>
+      <c r="B385" s="14"/>
+      <c r="C385" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="D385" s="10"/>
+    </row>
+    <row r="386" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A386" s="43"/>
+      <c r="B386" s="14"/>
+      <c r="C386" s="15"/>
+      <c r="D386" s="10"/>
+    </row>
+    <row r="387" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A387" s="43"/>
+      <c r="B387" s="14"/>
+      <c r="C387" s="15"/>
+      <c r="D387" s="10"/>
+    </row>
+    <row r="388" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A388" s="43"/>
+      <c r="B388" s="14"/>
+      <c r="C388" s="15"/>
+      <c r="D388" s="10"/>
+    </row>
+    <row r="389" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A389" s="43"/>
+      <c r="B389" s="14"/>
+      <c r="C389" s="15"/>
+      <c r="D389" s="10"/>
+    </row>
+    <row r="390" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A390" s="43"/>
+      <c r="B390" s="14"/>
+      <c r="C390" s="15"/>
+      <c r="D390" s="10"/>
+    </row>
+    <row r="391" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A391" s="43"/>
+      <c r="B391" s="14"/>
+      <c r="C391" s="15"/>
+      <c r="D391" s="10"/>
+    </row>
+    <row r="392" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A392" s="43"/>
+      <c r="B392" s="44"/>
+      <c r="C392" s="15"/>
+      <c r="D392" s="45"/>
+    </row>
+    <row r="393" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A393" s="43"/>
+      <c r="B393" s="46"/>
+      <c r="C393" s="15"/>
+      <c r="D393" s="45"/>
+    </row>
+    <row r="394" ht="52.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A394" s="43"/>
+      <c r="B394" s="47"/>
+      <c r="C394" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="D394" s="2"/>
+    </row>
+    <row r="395" ht="18.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A395" s="43"/>
+      <c r="B395" s="44"/>
+      <c r="C395" s="15"/>
+      <c r="D395" s="2"/>
+    </row>
+    <row r="396" ht="38.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A396" s="43"/>
+      <c r="B396" s="46"/>
+      <c r="C396" s="15"/>
+      <c r="D396" s="2"/>
+    </row>
+    <row r="397" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A397" s="39" t="s">
+        <v>285</v>
+      </c>
+      <c r="B397" s="47"/>
+      <c r="C397" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D379" s="2"/>
-    </row>
-    <row r="380" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A380" s="39"/>
-      <c r="B380" s="44"/>
-      <c r="C380" s="15"/>
-      <c r="D380" s="45"/>
-    </row>
-    <row r="381" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A381" s="39"/>
-      <c r="B381" s="44"/>
-      <c r="C381" s="15"/>
-      <c r="D381" s="45"/>
-    </row>
-    <row r="382" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A382" s="39"/>
-      <c r="B382" s="44"/>
-      <c r="C382" s="15"/>
-      <c r="D382" s="2"/>
-    </row>
-    <row r="383" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A383" s="39"/>
-      <c r="B383" s="46"/>
-      <c r="C383" s="15"/>
-      <c r="D383" s="2"/>
+      <c r="D397" s="2"/>
+    </row>
+    <row r="398" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A398" s="39"/>
+      <c r="B398" s="44"/>
+      <c r="C398" s="15"/>
+      <c r="D398" s="45"/>
+    </row>
+    <row r="399" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A399" s="39"/>
+      <c r="B399" s="44"/>
+      <c r="C399" s="15"/>
+      <c r="D399" s="45"/>
+    </row>
+    <row r="400" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A400" s="39"/>
+      <c r="B400" s="44"/>
+      <c r="C400" s="15"/>
+      <c r="D400" s="2"/>
+    </row>
+    <row r="401" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A401" s="39"/>
+      <c r="B401" s="46"/>
+      <c r="C401" s="15"/>
+      <c r="D401" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="98">
@@ -7481,96 +7679,96 @@
     <mergeCell ref="C16:C20"/>
     <mergeCell ref="C21:C29"/>
     <mergeCell ref="C30:C32"/>
-    <mergeCell ref="A33:A67"/>
+    <mergeCell ref="A33:A72"/>
     <mergeCell ref="C33:C35"/>
     <mergeCell ref="C36:C41"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C56:C58"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="C61:C64"/>
-    <mergeCell ref="B65:B68"/>
-    <mergeCell ref="C65:C67"/>
-    <mergeCell ref="A68:A91"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="B70:B72"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="C75:C79"/>
+    <mergeCell ref="C42:C48"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="C70:C72"/>
+    <mergeCell ref="A73:A96"/>
+    <mergeCell ref="C74:C79"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B78:B80"/>
     <mergeCell ref="C80:C84"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="C87:C90"/>
-    <mergeCell ref="A92:A96"/>
-    <mergeCell ref="C92:C94"/>
-    <mergeCell ref="C95:C96"/>
-    <mergeCell ref="A97:A114"/>
+    <mergeCell ref="C85:C89"/>
+    <mergeCell ref="C90:C91"/>
+    <mergeCell ref="C92:C95"/>
+    <mergeCell ref="A97:A101"/>
     <mergeCell ref="C97:C99"/>
-    <mergeCell ref="B98:B99"/>
-    <mergeCell ref="B100:B101"/>
     <mergeCell ref="C100:C101"/>
-    <mergeCell ref="B102:B103"/>
-    <mergeCell ref="C102:C114"/>
+    <mergeCell ref="A102:A119"/>
+    <mergeCell ref="C102:C104"/>
+    <mergeCell ref="B103:B104"/>
+    <mergeCell ref="B105:B106"/>
+    <mergeCell ref="C105:C106"/>
     <mergeCell ref="B107:B108"/>
-    <mergeCell ref="B109:B110"/>
-    <mergeCell ref="B111:B112"/>
-    <mergeCell ref="B115:B116"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B125:B126"/>
-    <mergeCell ref="B128:B135"/>
-    <mergeCell ref="B136:B137"/>
-    <mergeCell ref="B138:B139"/>
-    <mergeCell ref="B140:B142"/>
-    <mergeCell ref="B143:B144"/>
-    <mergeCell ref="B145:B146"/>
-    <mergeCell ref="B147:B149"/>
-    <mergeCell ref="B152:B154"/>
-    <mergeCell ref="B156:B160"/>
-    <mergeCell ref="B162:B163"/>
+    <mergeCell ref="C107:C119"/>
+    <mergeCell ref="B112:B113"/>
+    <mergeCell ref="B114:B115"/>
+    <mergeCell ref="B116:B117"/>
+    <mergeCell ref="B120:B121"/>
+    <mergeCell ref="B127:B129"/>
+    <mergeCell ref="B135:B136"/>
+    <mergeCell ref="B138:B145"/>
+    <mergeCell ref="B146:B147"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="B150:B152"/>
+    <mergeCell ref="B153:B154"/>
+    <mergeCell ref="B155:B156"/>
+    <mergeCell ref="B157:B159"/>
+    <mergeCell ref="B162:B164"/>
     <mergeCell ref="B166:B170"/>
     <mergeCell ref="B172:B173"/>
     <mergeCell ref="B176:B180"/>
-    <mergeCell ref="B185:B188"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="B195:B265"/>
-    <mergeCell ref="B267:B268"/>
-    <mergeCell ref="B269:B270"/>
-    <mergeCell ref="B271:B272"/>
-    <mergeCell ref="B273:B274"/>
-    <mergeCell ref="B275:B279"/>
-    <mergeCell ref="A280:A281"/>
-    <mergeCell ref="C280:C281"/>
-    <mergeCell ref="A282:A297"/>
-    <mergeCell ref="C282:C283"/>
-    <mergeCell ref="C284:C292"/>
-    <mergeCell ref="C293:C297"/>
-    <mergeCell ref="A298:A339"/>
-    <mergeCell ref="C298:C302"/>
-    <mergeCell ref="C303:C308"/>
-    <mergeCell ref="C309:C310"/>
-    <mergeCell ref="C311:C313"/>
-    <mergeCell ref="C314:C315"/>
-    <mergeCell ref="C316:C318"/>
-    <mergeCell ref="C320:C325"/>
-    <mergeCell ref="C326:C339"/>
-    <mergeCell ref="A340:A349"/>
-    <mergeCell ref="C340:C347"/>
-    <mergeCell ref="C348:C349"/>
-    <mergeCell ref="A350:A355"/>
-    <mergeCell ref="C350:C355"/>
-    <mergeCell ref="A356:A362"/>
-    <mergeCell ref="C356:C362"/>
-    <mergeCell ref="A363:A366"/>
-    <mergeCell ref="C363:C366"/>
-    <mergeCell ref="A367:A378"/>
-    <mergeCell ref="C367:C375"/>
-    <mergeCell ref="C376:C378"/>
-    <mergeCell ref="A379:A383"/>
-    <mergeCell ref="C379:C383"/>
+    <mergeCell ref="B182:B183"/>
+    <mergeCell ref="B186:B190"/>
+    <mergeCell ref="B195:B198"/>
+    <mergeCell ref="B200:B203"/>
+    <mergeCell ref="B205:B275"/>
+    <mergeCell ref="B277:B278"/>
+    <mergeCell ref="B279:B280"/>
+    <mergeCell ref="B281:B282"/>
+    <mergeCell ref="B283:B284"/>
+    <mergeCell ref="B289:B293"/>
+    <mergeCell ref="A298:A299"/>
+    <mergeCell ref="C298:C299"/>
+    <mergeCell ref="A300:A315"/>
+    <mergeCell ref="C300:C301"/>
+    <mergeCell ref="C302:C310"/>
+    <mergeCell ref="C311:C315"/>
+    <mergeCell ref="A316:A357"/>
+    <mergeCell ref="C316:C320"/>
+    <mergeCell ref="C321:C326"/>
+    <mergeCell ref="C327:C328"/>
+    <mergeCell ref="C329:C331"/>
+    <mergeCell ref="C332:C333"/>
+    <mergeCell ref="C334:C336"/>
+    <mergeCell ref="C338:C343"/>
+    <mergeCell ref="C344:C357"/>
+    <mergeCell ref="A358:A367"/>
+    <mergeCell ref="C358:C365"/>
+    <mergeCell ref="C366:C367"/>
+    <mergeCell ref="A368:A373"/>
+    <mergeCell ref="C368:C373"/>
+    <mergeCell ref="A374:A380"/>
+    <mergeCell ref="C374:C380"/>
+    <mergeCell ref="A381:A384"/>
+    <mergeCell ref="C381:C384"/>
+    <mergeCell ref="A385:A396"/>
+    <mergeCell ref="C385:C393"/>
+    <mergeCell ref="C394:C396"/>
+    <mergeCell ref="A397:A401"/>
+    <mergeCell ref="C397:C401"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7588,7 +7786,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="48" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
       <c r="B1" s="48"/>
       <c r="C1" s="48"/>
@@ -7616,15 +7814,15 @@
     </row>
     <row r="3" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="49" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C3" s="49"/>
       <c r="D3" s="49"/>
       <c r="E3" s="49" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="F3" s="49"/>
       <c r="G3" s="49"/>
@@ -7636,39 +7834,39 @@
     <row r="4" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="49"/>
       <c r="B4" s="50" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="C4" s="50" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="D4" s="50" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
       <c r="E4" s="50" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="F4" s="50" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="G4" s="50" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="H4" s="50" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="I4" s="50" t="s">
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="J4" s="50" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="K4" s="50" t="s">
-        <v>279</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="51" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
       <c r="B5" s="52"/>
       <c r="C5" s="52"/>
@@ -7839,7 +8037,7 @@
     </row>
     <row r="18" ht="70" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="55" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="B18" s="56"/>
       <c r="C18" s="56"/>
@@ -7919,7 +8117,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="57" t="s">
-        <v>282</v>
+        <v>300</v>
       </c>
       <c r="B1" s="57"/>
       <c r="C1" s="57"/>
@@ -7932,36 +8130,36 @@
     </row>
     <row r="2" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="58" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
       <c r="B2" s="59" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="C2" s="59" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="D2" s="59" t="s">
-        <v>285</v>
+        <v>303</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>286</v>
+        <v>304</v>
       </c>
       <c r="F2" s="59" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="G2" s="59" t="s">
-        <v>288</v>
+        <v>306</v>
       </c>
       <c r="H2" s="59" t="s">
-        <v>289</v>
+        <v>307</v>
       </c>
       <c r="I2" s="59" t="s">
-        <v>290</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="60" t="s">
-        <v>291</v>
+        <v>309</v>
       </c>
       <c r="B3" s="61"/>
       <c r="C3" s="61"/>
@@ -8073,7 +8271,7 @@
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="60" t="s">
-        <v>292</v>
+        <v>310</v>
       </c>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -8160,7 +8358,7 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="63" t="s">
-        <v>293</v>
+        <v>311</v>
       </c>
       <c r="B1" s="63"/>
       <c r="C1" s="63"/>
@@ -8168,21 +8366,21 @@
     </row>
     <row r="2" ht="60" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="65" t="s">
-        <v>291</v>
+        <v>309</v>
       </c>
       <c r="B3" s="65"/>
       <c r="C3" s="65"/>
@@ -8238,7 +8436,7 @@
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="65" t="s">
-        <v>292</v>
+        <v>310</v>
       </c>
       <c r="B12" s="65"/>
       <c r="C12" s="65"/>
@@ -8297,7 +8495,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -8305,16 +8503,16 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>298</v>
+        <v>316</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -8386,7 +8584,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
-        <v>302</v>
+        <v>320</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -8394,16 +8592,16 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="D2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -8463,7 +8661,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
-        <v>304</v>
+        <v>322</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -8472,10 +8670,10 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
       <c r="B2" s="71" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="C2" s="71">
         <v>2025</v>
@@ -8484,7 +8682,7 @@
         <v>2024</v>
       </c>
       <c r="E2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -8528,7 +8726,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="76" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
       <c r="B1" s="76"/>
       <c r="C1" s="76"/>
@@ -8536,14 +8734,14 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
       <c r="C2" s="64"/>
       <c r="D2" s="64" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>